<commit_message>
Add 90-day run results: 12 new relevant items, replies for 10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015dXgfxu1ugCxsD9bCGxkqs
</commit_message>
<xml_diff>
--- a/lynkk-reddit-leads/results/2026-10-11/engagement_replies_2026-10-11.xlsx
+++ b/lynkk-reddit-leads/results/2026-10-11/engagement_replies_2026-10-11.xlsx
@@ -427,20 +427,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
     <col width="35" customWidth="1" min="8" max="8"/>
     <col width="70" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1490,6 +1490,104 @@
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="n">
         <v>53</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/AIAssisted/comments/1x36z0d/whats_the_most_useful_thing_your_ai_recorder/</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/AIAssisted/comments/1x36z0d/whats_the_most_useful_thing_your_ai_recorder/</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>r/AIAssisted</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>u/Comfortable-Pay611</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>What’s the most useful thing your AI recorder gives you after a meeting?</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Discussion about which AI recorder output people actually use.</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>A follow-up that's basically ready to send wins for most people, but only if it's built from the action items rather than the summary. The summary is for whoever missed the meeting; the action items with owners and dates are what you actually send to the client. Asking for 'decisions, action items with owner and date, and open questions' as the output shape gets you most of the way to that email.</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/ConstructionManagers/comments/1vm1lxg/what_tools_help_you_be_more_efficient_and/</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/ConstructionManagers/comments/1vm1lxg/what_tools_help_you_be_more_efficient_and/</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>r/ConstructionManagers</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>u/Bobcatbob9</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>What tools help you be more efficient and effective as a PM.</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Construction PM on four projects asking what tools help; meeting minutes is one concrete win.</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Meeting minutes is the easiest one to take off your plate first. Record the OAC and sub meetings (with permission), let a tool draft minutes with action items, owners and dates, then spend five minutes correcting it before it goes out. That alone usually gives back a few hours a week. Copilot can help with drafting submittal logs and emails if you already have it. Congrats on the newborn, and protect that time off.</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="n">
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1534,6 +1632,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>